<commit_message>
Isıtma hesapları: kullanıcının projesindeki 5x110 kW kazan ve ekipmanlarla; çizime dokunulmaz
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/isitma_944_343/ISITMA_HESAPLARI.xlsx
+++ b/proje/isitma_944_343/ISITMA_HESAPLARI.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B69"/>
+  <dimension ref="A1:B67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -693,7 +693,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>2 adet</t>
+          <t>5 adet</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>65 kW</t>
+          <t>110 kW</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>2 × 65 = 130 kW (111.800 kcal/h)</t>
+          <t>5 × 110 = 550 kW (473.000 kcal/h)</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>65 / (1,163 × 20) = 2,79 m³/h (kazan başına)</t>
+          <t>110 / (1,163 × 20) = 4,73 m³/h (kazan başına)</t>
         </is>
       </c>
     </row>
@@ -767,19 +767,19 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>3,00 m³/h - 6,0 mSS (kazan başına)</t>
+          <t>5,00 m³/h - 5,0 mSS (kazan başına)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Q sistem = Q ısı kaybı / (1,163 × ΔT)</t>
+          <t>Q sistem = Q radyatör / (1,163 × ΔT)</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>86,04 / (1,163 × 20) = 3,70 m³/h</t>
+          <t>461,1 / (1,163 × 20) = 19,82 m³/h</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>4,50 m³/h (≥ 3,70 × 1,10)</t>
+          <t>20,00 m³/h - 10,0 mSS</t>
         </is>
       </c>
     </row>
@@ -882,7 +882,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>7,0 mSS</t>
+          <t>10,0 mSS</t>
         </is>
       </c>
     </row>
@@ -903,237 +903,213 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Radyatör su hacmi</t>
+          <t>Toplam sistem su hacmi (V_s)</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>222,0 m × 5,7 l/m = 1.265 Litre</t>
+          <t>550 kW × 10 lt/kW = 5.500 Litre</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Toplam sistem su hacmi (V_s) (+%30 tesisat)</t>
+          <t>Genleşme katsayısı (e) — 90 °C</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>1.645 Litre</t>
+          <t>0,0359</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Genleşme katsayısı (e) — 90 °C</t>
+          <t>Genleşen su hacmi (V_e)</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>0,0359</t>
+          <t>5.500 × 0,0359 = 197,5 Litre</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Genleşen su hacmi (V_e)</t>
+          <t>Yedek su hacmi (V_WR) — %0,5</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>1.645 × 0,0359 = 59,1 Litre</t>
+          <t>27,5 Litre</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Yedek su hacmi (V_WR) — %0,5</t>
+          <t>Statik yükseklik (H_statik)</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>8,2 Litre</t>
+          <t>24 m</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Statik yükseklik (H_statik)</t>
+          <t>Ön basınç (P_0) = H/10 + 0,3</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>24 m</t>
+          <t>2,7 bar</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Ön basınç (P_0) = H/10 + 0,3</t>
+          <t>Emniyet ventili açma basıncı (P_sv)</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>2,7 bar</t>
+          <t>6,0 bar</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Emniyet ventili açma basıncı (P_sv)</t>
+          <t>Son basınç (P_e) = P_sv − 0,5</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>6,0 bar</t>
+          <t>5,5 bar</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Son basınç (P_e) = P_sv − 0,5</t>
+          <t>Gerekli nominal hacim V_n = (V_e+V_WR)·(P_e+1)/(P_e−P_0)</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>5,5 bar</t>
+          <t>522 Litre</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Gerekli nominal hacim V_n = (V_e+V_WR)·(P_e+1)/(P_e−P_0)</t>
+          <t>Seçilen tank (GT-01)</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>156 Litre</t>
+          <t>1000 Litre</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>Seçilen tank (GT-01)</t>
-        </is>
-      </c>
-      <c r="B58" s="5" t="inlineStr">
-        <is>
-          <t>200 Litre</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="6" t="inlineStr">
-        <is>
-          <t>Sonuç: Seçilen 200 litre genleşme deposu yeterlidir.</t>
+      <c r="A58" s="6" t="inlineStr">
+        <is>
+          <t>Sonuç: Seçilen 1000 litre genleşme deposu yeterlidir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>7. DENGE KABI BOYUTLANDIRMA HESABI (DK-01)</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>7. DENGE KABI BOYUTLANDIRMA HESABI (DK-01)</t>
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Maksimum sistem debisi (Q_maks)</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>23,65 m³/h = 0,00657 m³/s</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>Maksimum sistem debisi (Q_maks)</t>
+          <t>Azami gövde akış hızı (v)</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>5,59 m³/h = 0,00155 m³/s</t>
+          <t>0,15 m/s</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Azami gövde akış hızı (v)</t>
+          <t>Hesaplanan iç çap D = √[4·Q/(π·v)]</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>0,15 m/s</t>
+          <t>236 mm</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>Hesaplanan iç çap D = √[4·Q/(π·v)]</t>
+          <t>Seçilen denge kabı iç çapı</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>115 mm</t>
+          <t>Ø 300 mm</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Seçilen denge kabı iç çapı</t>
+          <t>Denge kabı ısıl yükü</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Ø 150 mm</t>
+          <t>550 kW</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>Denge kabı ısıl yükü</t>
+          <t>Giriş – çıkış çapları</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>130 kW</t>
+          <t>DN100 (4")</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>Denge kabı yüksekliği</t>
-        </is>
-      </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>900 mm</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>Giriş – çıkış çapları</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>DN50</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="6" t="inlineStr">
-        <is>
-          <t>Sonuç: Seçilen Ø150 mm denge kabı yeterlidir.</t>
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>Sonuç: Seçilen Ø300 mm denge kabı yeterlidir.</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1167,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>130 kW</t>
+          <t>550 kW</t>
         </is>
       </c>
     </row>
@@ -1229,7 +1205,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A_alt = 130 × 6 = 780 cm²</t>
+          <t>A_alt = 550 × 6 = 3.300 cm²</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1217,7 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>30 × 30 cm  (900 cm²)</t>
+          <t>60 × 60 cm  (3.600 cm²)</t>
         </is>
       </c>
     </row>
@@ -1253,14 +1229,14 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Ø320 mm  (804 cm²)</t>
+          <t>Ø700 mm  (3.848 cm²)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Sonuç: Seçilen alt havalandırma menfezi: 30 × 30 cm.</t>
+          <t>Sonuç: Seçilen alt havalandırma menfezi: 60 × 60 cm.</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1250,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>A_üst = 130 × 3 = 390 cm²</t>
+          <t>A_üst = 550 × 3 = 1.650 cm²</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1262,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>20 × 20 cm  (400 cm²)</t>
+          <t>45 × 40 cm  (1.800 cm²)</t>
         </is>
       </c>
     </row>
@@ -1298,14 +1274,14 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Ø250 mm  (491 cm²)</t>
+          <t>Ø500 mm  (1.963 cm²)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Sonuç: Seçilen üst havalandırma menfezi: 20 × 20 cm.</t>
+          <t>Sonuç: Seçilen üst havalandırma menfezi: 45 × 40 cm.</t>
         </is>
       </c>
     </row>
@@ -1441,10 +1417,10 @@
         </is>
       </c>
       <c r="E3" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>65</v>
+        <v>110</v>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
@@ -1534,17 +1510,17 @@
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>3,00</t>
+          <t>5,00</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>6,0</t>
+          <t>5,0</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>0,09</t>
+          <t>0,12</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -1553,7 +1529,7 @@
         </is>
       </c>
       <c r="H8" s="9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
@@ -1579,17 +1555,17 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>4,50</t>
+          <t>20,00</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>7,0</t>
+          <t>10,0</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>0,15</t>
+          <t>1,10</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
@@ -1665,20 +1641,20 @@
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>130</v>
+        <v>550</v>
       </c>
       <c r="D14" s="9" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>900</v>
+        <v>145</v>
       </c>
       <c r="F14" s="9" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>5,59</t>
+          <t>23,65</t>
         </is>
       </c>
       <c r="H14" s="9" t="n">
@@ -1746,7 +1722,7 @@
         </is>
       </c>
       <c r="D19" s="9" t="n">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
@@ -1823,14 +1799,14 @@
         </is>
       </c>
       <c r="D24" s="9" t="n">
-        <v>200</v>
+        <v>750</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>1"</t>
+          <t>1 1/2"</t>
         </is>
       </c>
       <c r="G24" s="9" t="n">

</xml_diff>

<commit_message>
Isıtma hesaplar: projede olmayan ekipman tabloları çıkarıldı, genel bilgiler tablo düzeni
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwXcqZmf9VPBpDgb8LPkn3
</commit_message>
<xml_diff>
--- a/proje/isitma_944_343/ISITMA_HESAPLARI.xlsx
+++ b/proje/isitma_944_343/ISITMA_HESAPLARI.xlsx
@@ -1327,7 +1327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1735,225 +1735,6 @@
         </is>
       </c>
       <c r="G19" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>NÖTRALİZASYON TANKI TABLOSU</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>CİHAZ NO</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>TANIMLAMA</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>CİHAZIN BULUNDUĞU YER</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>KAPASİTESİ (kW)</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>DEBİ (L/h)</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="inlineStr">
-        <is>
-          <t>GİRİŞ ÇIKIŞ ÇAPI (")</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>ADET</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>NT-01</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>NÖTRALİZASYON TANKI</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>BODRUM</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="n">
-        <v>750</v>
-      </c>
-      <c r="E24" s="9" t="n">
-        <v>100</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>1 1/2"</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>KAZAN BESLEME</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>CİHAZ NO</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>TANIMLAMA</t>
-        </is>
-      </c>
-      <c r="C28" s="8" t="inlineStr">
-        <is>
-          <t>CİHAZIN BULUNDUĞU YER</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>ÇAP (mm)</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>ADET</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>KB-1</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>MEKANİK KAZAN BESLEME</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>BODRUM</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="n">
-        <v>25</v>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>SU YUMUŞATMA CİHAZI</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>CİHAZ NO</t>
-        </is>
-      </c>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>TİP</t>
-        </is>
-      </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>HİZMET ETTİĞİ ALAN</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>KAPASİTE (m³/h)</t>
-        </is>
-      </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>İŞLETME BASINCI (bar)</t>
-        </is>
-      </c>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>REÇİNE MİKTARI (lt)</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>GİRİŞ - ÇIKIŞ ÇAPI</t>
-        </is>
-      </c>
-      <c r="H33" s="8" t="inlineStr">
-        <is>
-          <t>ADET</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>SYC-1</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>TANDEMLİ VOLUMETRİK SU YUMUŞATMA CİHAZI</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
-        <is>
-          <t>ISITMA SİSTEMİ</t>
-        </is>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>1,5</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>2,5-7,5</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>1"-1"</t>
-        </is>
-      </c>
-      <c r="H34" s="9" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>